<commit_message>
Phase 2: remove features outside the refocused scope
The platform now centres on security, institution data submission and
verification. Removed:
- ghost-cluster graph detector, its endpoints, screens and Cytoscape deps
- risk score, risk leaderboard, inspection shortlist, IsolationForest
  STATISTICAL_ANOMALY (and the supernumerary-share signal, scenario K)
- SEQUENTIAL_APAAR, LAST_MINUTE_BULK and PHANTOM_PROGRESSION detectors
- the student confirm/dispute flow; corrections stay and now raise
  STUDENT_CORRECTION
- the compliance certificate, the non-reporting tracker and reminders
- admin load-scenario and run-detectors (reseed and audit check stay)
- seed scenarios B, G, H, I, K, their ground truth, tests and eval rows

Also fixes a latent bug in scenario A: the TFW-over-cap case ignored TFW
entrants already in the base cohort, so the expected excess could be off
by one.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/sample_1_excess_intake.xlsx
+++ b/samples/sample_1_excess_intake.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P87"/>
+  <dimension ref="A1:P67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -563,7 +563,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -645,7 +645,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -727,7 +727,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -809,7 +809,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -891,7 +891,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -973,7 +973,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1137,7 +1137,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1301,7 +1301,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1647,7 +1647,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1729,7 +1729,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1893,7 +1893,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1975,7 +1975,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -2057,7 +2057,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -2221,7 +2221,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -2549,7 +2549,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -2631,7 +2631,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -2713,7 +2713,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -2795,7 +2795,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -2877,7 +2877,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -2959,7 +2959,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -3041,7 +3041,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -3205,7 +3205,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -3287,7 +3287,7 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
@@ -3369,7 +3369,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -3451,7 +3451,7 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
@@ -3533,7 +3533,7 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
@@ -3797,7 +3797,7 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
@@ -3879,7 +3879,7 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
@@ -3961,7 +3961,7 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
@@ -4125,7 +4125,7 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
@@ -4207,7 +4207,7 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
@@ -4289,7 +4289,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -4371,7 +4371,7 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
@@ -4453,7 +4453,7 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
@@ -4535,7 +4535,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
@@ -4617,7 +4617,7 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
@@ -4699,7 +4699,7 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
@@ -4781,7 +4781,7 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
@@ -4863,7 +4863,7 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
@@ -4945,7 +4945,7 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
@@ -5027,7 +5027,7 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
@@ -5109,7 +5109,7 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
@@ -5191,7 +5191,7 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
@@ -5273,7 +5273,7 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
@@ -5355,7 +5355,7 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
@@ -5437,7 +5437,7 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
@@ -5519,7 +5519,7 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
@@ -5601,7 +5601,7 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
@@ -5713,1666 +5713,26 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>372693176556</t>
-        </is>
-      </c>
+      <c r="A67" t="inlineStr"/>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Sneha Iyer</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>15-05-2004</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>OBC-NCL</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>indian</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>+91 76976 92903</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>student63@example.invalid</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>08345324306</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>B.Tech</t>
-        </is>
-      </c>
-      <c r="K67" t="inlineStr">
-        <is>
-          <t>Civil Engineering</t>
-        </is>
-      </c>
-      <c r="L67" t="inlineStr">
-        <is>
-          <t>2026-2027</t>
-        </is>
-      </c>
-      <c r="M67" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N67" t="inlineStr">
-        <is>
-          <t>Regular</t>
-        </is>
-      </c>
-      <c r="O67" t="inlineStr">
-        <is>
-          <t>15.07.2026</t>
-        </is>
-      </c>
-      <c r="P67" t="inlineStr">
-        <is>
-          <t>Admitted</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>410570826663</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>Arjun Nair</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>16-07-2008</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>SC</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>INDIAN</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>+91 79314 44584</t>
-        </is>
-      </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>student64@example.invalid</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>07809642225</t>
-        </is>
-      </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>B.Tech</t>
-        </is>
-      </c>
-      <c r="K68" t="inlineStr">
-        <is>
-          <t>Civil Engineering</t>
-        </is>
-      </c>
-      <c r="L68" t="inlineStr">
-        <is>
-          <t>2026-27</t>
-        </is>
-      </c>
-      <c r="M68" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N68" t="inlineStr">
-        <is>
-          <t>Regular</t>
-        </is>
-      </c>
-      <c r="O68" t="inlineStr">
-        <is>
-          <t>26-08-2026</t>
-        </is>
-      </c>
-      <c r="P68" t="inlineStr">
-        <is>
-          <t>Admitted</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>688907959686</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>Priya Menon</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>2004-04-11</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>obc</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>Indian</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>+91 97506 18045</t>
-        </is>
-      </c>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>student65@example.invalid</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>09311242529</t>
-        </is>
-      </c>
-      <c r="J69" t="inlineStr">
-        <is>
-          <t>B.Tech</t>
-        </is>
-      </c>
-      <c r="K69" t="inlineStr">
-        <is>
-          <t>Civil Engineering</t>
-        </is>
-      </c>
-      <c r="L69" t="inlineStr">
-        <is>
-          <t>2026-27</t>
-        </is>
-      </c>
-      <c r="M69" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N69" t="inlineStr">
-        <is>
-          <t>Regular</t>
-        </is>
-      </c>
-      <c r="O69" t="inlineStr">
-        <is>
-          <t>07-09-2026</t>
-        </is>
-      </c>
-      <c r="P69" t="inlineStr">
-        <is>
-          <t>Admitted</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>489574942730</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>Rohit Verma</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>10.07.2008</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>EWS</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>INDIAN</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>+91 93345 47802</t>
-        </is>
-      </c>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>student66@example.invalid</t>
-        </is>
-      </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>09250449560</t>
-        </is>
-      </c>
-      <c r="J70" t="inlineStr">
-        <is>
-          <t>B.Tech</t>
-        </is>
-      </c>
-      <c r="K70" t="inlineStr">
-        <is>
-          <t>Civil Engineering</t>
-        </is>
-      </c>
-      <c r="L70" t="inlineStr">
-        <is>
-          <t>2026-27</t>
-        </is>
-      </c>
-      <c r="M70" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N70" t="inlineStr">
-        <is>
-          <t>REGULAR</t>
-        </is>
-      </c>
-      <c r="O70" t="inlineStr">
-        <is>
-          <t>17-08-2026</t>
-        </is>
-      </c>
-      <c r="P70" t="inlineStr">
-        <is>
-          <t>admitted</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>259665633768</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>Fatima Shaikh</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>22-04-2008</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>indian</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>+91 96828 22515</t>
-        </is>
-      </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>student67@example.invalid</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>09226794717</t>
-        </is>
-      </c>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>B.Tech</t>
-        </is>
-      </c>
-      <c r="K71" t="inlineStr">
-        <is>
-          <t>Civil Engineering</t>
-        </is>
-      </c>
-      <c r="L71" t="inlineStr">
-        <is>
-          <t>2026-27</t>
-        </is>
-      </c>
-      <c r="M71" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N71" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
-      <c r="O71" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="P71" t="inlineStr">
-        <is>
-          <t>admitted</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>466017347670</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>Karthik Reddy</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>23/09/2005</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>SC</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>indian</t>
-        </is>
-      </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>+91 80183 21473</t>
-        </is>
-      </c>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>student68@example.invalid</t>
-        </is>
-      </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>08924270785</t>
-        </is>
-      </c>
-      <c r="J72" t="inlineStr">
-        <is>
-          <t>B.Tech</t>
-        </is>
-      </c>
-      <c r="K72" t="inlineStr">
-        <is>
-          <t>Civil Engineering</t>
-        </is>
-      </c>
-      <c r="L72" t="inlineStr">
-        <is>
-          <t>2026-27</t>
-        </is>
-      </c>
-      <c r="M72" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N72" t="inlineStr">
-        <is>
-          <t>REGULAR</t>
-        </is>
-      </c>
-      <c r="O72" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="P72" t="inlineStr">
-        <is>
-          <t>Admitted</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>223018514600</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>Neha Gupta</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>22.04.2004</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>SC</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>Indian</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>+91 84017 25403</t>
-        </is>
-      </c>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>student69@example.invalid</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>08528173370</t>
-        </is>
-      </c>
-      <c r="J73" t="inlineStr">
-        <is>
-          <t>B.Tech</t>
-        </is>
-      </c>
-      <c r="K73" t="inlineStr">
-        <is>
-          <t>Civil Engineering</t>
-        </is>
-      </c>
-      <c r="L73" t="inlineStr">
-        <is>
-          <t>2026-2027</t>
-        </is>
-      </c>
-      <c r="M73" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N73" t="inlineStr">
-        <is>
-          <t>REGULAR</t>
-        </is>
-      </c>
-      <c r="O73" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="P73" t="inlineStr">
-        <is>
-          <t>Admitted</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>774856838093</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>Imran Qureshi</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>04.01.2004</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>OBC-NCL</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>indian</t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>+91 74637 71569</t>
-        </is>
-      </c>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>student70@example.invalid</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>08631063987</t>
-        </is>
-      </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>B.Tech</t>
-        </is>
-      </c>
-      <c r="K74" t="inlineStr">
-        <is>
-          <t>Civil Engineering</t>
-        </is>
-      </c>
-      <c r="L74" t="inlineStr">
-        <is>
-          <t>2026-27</t>
-        </is>
-      </c>
-      <c r="M74" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N74" t="inlineStr">
-        <is>
-          <t>Regular</t>
-        </is>
-      </c>
-      <c r="O74" t="inlineStr">
-        <is>
-          <t>06-08-2026</t>
-        </is>
-      </c>
-      <c r="P74" t="inlineStr">
-        <is>
-          <t>Admitted</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>634592634699</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>Divya Pillai</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>female</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>11-01-2004</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>obc</t>
-        </is>
-      </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>INDIAN</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>+91 74713 17850</t>
-        </is>
-      </c>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>student71@example.invalid</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>07741725082</t>
-        </is>
-      </c>
-      <c r="J75" t="inlineStr">
-        <is>
-          <t>B.Tech</t>
-        </is>
-      </c>
-      <c r="K75" t="inlineStr">
-        <is>
-          <t>Civil Engineering</t>
-        </is>
-      </c>
-      <c r="L75" t="inlineStr">
-        <is>
-          <t>2026-27</t>
-        </is>
-      </c>
-      <c r="M75" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N75" t="inlineStr">
-        <is>
-          <t>REGULAR</t>
-        </is>
-      </c>
-      <c r="O75" t="inlineStr">
-        <is>
-          <t>09/09/2026</t>
-        </is>
-      </c>
-      <c r="P75" t="inlineStr">
-        <is>
-          <t>Admitted</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>427691334219</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>Sandeep Yadav</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>2006-05-02</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>EWS</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>Indian</t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>+91 99264 60220</t>
-        </is>
-      </c>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>student72@example.invalid</t>
-        </is>
-      </c>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>09399812805</t>
-        </is>
-      </c>
-      <c r="J76" t="inlineStr">
-        <is>
-          <t>B.Tech</t>
-        </is>
-      </c>
-      <c r="K76" t="inlineStr">
-        <is>
-          <t>Civil Engineering</t>
-        </is>
-      </c>
-      <c r="L76" t="inlineStr">
-        <is>
-          <t>2026-27</t>
-        </is>
-      </c>
-      <c r="M76" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N76" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
-      <c r="O76" t="inlineStr">
-        <is>
-          <t>07.06.2026</t>
-        </is>
-      </c>
-      <c r="P76" t="inlineStr">
-        <is>
-          <t>Admitted</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>957792614967</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>Meera Joshi</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>2008-04-22</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>GEN</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>Indian</t>
-        </is>
-      </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>+91 91292 95218</t>
-        </is>
-      </c>
-      <c r="H77" t="inlineStr">
-        <is>
-          <t>student73@example.invalid</t>
-        </is>
-      </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>08183630465</t>
-        </is>
-      </c>
-      <c r="J77" t="inlineStr">
-        <is>
-          <t>B.Tech</t>
-        </is>
-      </c>
-      <c r="K77" t="inlineStr">
-        <is>
-          <t>Civil Engineering</t>
-        </is>
-      </c>
-      <c r="L77" t="inlineStr">
-        <is>
-          <t>2026-27</t>
-        </is>
-      </c>
-      <c r="M77" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N77" t="inlineStr">
-        <is>
-          <t>Regular</t>
-        </is>
-      </c>
-      <c r="O77" t="inlineStr">
-        <is>
-          <t>30.07.2026</t>
-        </is>
-      </c>
-      <c r="P77" t="inlineStr">
-        <is>
-          <t>admitted</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>431668627350</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>Tarun Bose</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>19.07.2004</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>obc</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>indian</t>
-        </is>
-      </c>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>+91 93511 61283</t>
-        </is>
-      </c>
-      <c r="H78" t="inlineStr">
-        <is>
-          <t>student74@example.invalid</t>
-        </is>
-      </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>08021590930</t>
-        </is>
-      </c>
-      <c r="J78" t="inlineStr">
-        <is>
-          <t>B.Tech</t>
-        </is>
-      </c>
-      <c r="K78" t="inlineStr">
-        <is>
-          <t>Civil Engineering</t>
-        </is>
-      </c>
-      <c r="L78" t="inlineStr">
-        <is>
-          <t>2026-27</t>
-        </is>
-      </c>
-      <c r="M78" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N78" t="inlineStr">
-        <is>
-          <t>REGULAR</t>
-        </is>
-      </c>
-      <c r="O78" t="inlineStr">
-        <is>
-          <t>26-06-2026</t>
-        </is>
-      </c>
-      <c r="P78" t="inlineStr">
-        <is>
-          <t>Admitted</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>816562753200</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>Rahul Sharma</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>03/12/2005</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>SC</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>indian</t>
-        </is>
-      </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>+91 71454 17029</t>
-        </is>
-      </c>
-      <c r="H79" t="inlineStr">
-        <is>
-          <t>student75@example.invalid</t>
-        </is>
-      </c>
-      <c r="I79" t="inlineStr">
-        <is>
-          <t>08846666988</t>
-        </is>
-      </c>
-      <c r="J79" t="inlineStr">
-        <is>
-          <t>B.Tech</t>
-        </is>
-      </c>
-      <c r="K79" t="inlineStr">
-        <is>
-          <t>Civil Engineering</t>
-        </is>
-      </c>
-      <c r="L79" t="inlineStr">
-        <is>
-          <t>2026-27</t>
-        </is>
-      </c>
-      <c r="M79" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N79" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
-      <c r="O79" t="inlineStr">
-        <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="P79" t="inlineStr">
-        <is>
-          <t>admitted</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>425437956182</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>Aisha Khan</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>15.10.2008</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>INDIAN</t>
-        </is>
-      </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>+91 82652 23076</t>
-        </is>
-      </c>
-      <c r="H80" t="inlineStr">
-        <is>
-          <t>student76@example.invalid</t>
-        </is>
-      </c>
-      <c r="I80" t="inlineStr">
-        <is>
-          <t>08597068460</t>
-        </is>
-      </c>
-      <c r="J80" t="inlineStr">
-        <is>
-          <t>B.Tech</t>
-        </is>
-      </c>
-      <c r="K80" t="inlineStr">
-        <is>
-          <t>Civil Engineering</t>
-        </is>
-      </c>
-      <c r="L80" t="inlineStr">
-        <is>
-          <t>2026-27</t>
-        </is>
-      </c>
-      <c r="M80" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N80" t="inlineStr">
-        <is>
-          <t>REGULAR</t>
-        </is>
-      </c>
-      <c r="O80" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="P80" t="inlineStr">
-        <is>
-          <t>Admitted</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>445965346770</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>Vikram Patel</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>2004-02-23</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>EWS</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>indian</t>
-        </is>
-      </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>+91 76038 71851</t>
-        </is>
-      </c>
-      <c r="H81" t="inlineStr">
-        <is>
-          <t>student77@example.invalid</t>
-        </is>
-      </c>
-      <c r="I81" t="inlineStr">
-        <is>
-          <t>09117348339</t>
-        </is>
-      </c>
-      <c r="J81" t="inlineStr">
-        <is>
-          <t>B.Tech</t>
-        </is>
-      </c>
-      <c r="K81" t="inlineStr">
-        <is>
-          <t>Civil Engineering</t>
-        </is>
-      </c>
-      <c r="L81" t="inlineStr">
-        <is>
-          <t>2026-2027</t>
-        </is>
-      </c>
-      <c r="M81" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N81" t="inlineStr">
-        <is>
-          <t>Regular</t>
-        </is>
-      </c>
-      <c r="O81" t="inlineStr">
-        <is>
-          <t>22/06/2026</t>
-        </is>
-      </c>
-      <c r="P81" t="inlineStr">
-        <is>
-          <t>admitted</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>660348529498</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>Sneha Iyer</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>25/01/2007</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>SC</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>Indian</t>
-        </is>
-      </c>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>+91 80199 99446</t>
-        </is>
-      </c>
-      <c r="H82" t="inlineStr">
-        <is>
-          <t>student78@example.invalid</t>
-        </is>
-      </c>
-      <c r="I82" t="inlineStr">
-        <is>
-          <t>07474038401</t>
-        </is>
-      </c>
-      <c r="J82" t="inlineStr">
-        <is>
-          <t>B.Tech</t>
-        </is>
-      </c>
-      <c r="K82" t="inlineStr">
-        <is>
-          <t>Civil Engineering</t>
-        </is>
-      </c>
-      <c r="L82" t="inlineStr">
-        <is>
-          <t>2026-2027</t>
-        </is>
-      </c>
-      <c r="M82" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N82" t="inlineStr">
-        <is>
-          <t>Regular</t>
-        </is>
-      </c>
-      <c r="O82" t="inlineStr">
-        <is>
-          <t>01-07-2026</t>
-        </is>
-      </c>
-      <c r="P82" t="inlineStr">
-        <is>
-          <t>admitted</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>573167559469</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>Arjun Nair</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>female</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>2005-09-07</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>SC</t>
-        </is>
-      </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>INDIAN</t>
-        </is>
-      </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>+91 84148 81191</t>
-        </is>
-      </c>
-      <c r="H83" t="inlineStr">
-        <is>
-          <t>student79@example.invalid</t>
-        </is>
-      </c>
-      <c r="I83" t="inlineStr">
-        <is>
-          <t>07099651897</t>
-        </is>
-      </c>
-      <c r="J83" t="inlineStr">
-        <is>
-          <t>B.Tech</t>
-        </is>
-      </c>
-      <c r="K83" t="inlineStr">
-        <is>
-          <t>Civil Engineering</t>
-        </is>
-      </c>
-      <c r="L83" t="inlineStr">
-        <is>
-          <t>2026-2027</t>
-        </is>
-      </c>
-      <c r="M83" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N83" t="inlineStr">
-        <is>
-          <t>Regular</t>
-        </is>
-      </c>
-      <c r="O83" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="P83" t="inlineStr">
-        <is>
-          <t>admitted</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>527322515085</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>Priya Menon</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr">
-        <is>
-          <t>2007-09-26</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>GEN</t>
-        </is>
-      </c>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>Indian</t>
-        </is>
-      </c>
-      <c r="G84" t="inlineStr">
-        <is>
-          <t>+91 74844 35323</t>
-        </is>
-      </c>
-      <c r="H84" t="inlineStr">
-        <is>
-          <t>student80@example.invalid</t>
-        </is>
-      </c>
-      <c r="I84" t="inlineStr">
-        <is>
-          <t>08108405473</t>
-        </is>
-      </c>
-      <c r="J84" t="inlineStr">
-        <is>
-          <t>B.Tech</t>
-        </is>
-      </c>
-      <c r="K84" t="inlineStr">
-        <is>
-          <t>Civil Engineering</t>
-        </is>
-      </c>
-      <c r="L84" t="inlineStr">
-        <is>
-          <t>2026-27</t>
-        </is>
-      </c>
-      <c r="M84" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N84" t="inlineStr">
-        <is>
-          <t>REGULAR</t>
-        </is>
-      </c>
-      <c r="O84" t="inlineStr">
-        <is>
-          <t>23.07.2026</t>
-        </is>
-      </c>
-      <c r="P84" t="inlineStr">
-        <is>
-          <t>Admitted</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>212020554871</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>Rohit Verma</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>female</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>2004-07-06</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>OBC-NCL</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>indian</t>
-        </is>
-      </c>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>+91 85169 26461</t>
-        </is>
-      </c>
-      <c r="H85" t="inlineStr">
-        <is>
-          <t>student81@example.invalid</t>
-        </is>
-      </c>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t>08200356137</t>
-        </is>
-      </c>
-      <c r="J85" t="inlineStr">
-        <is>
-          <t>B.Tech</t>
-        </is>
-      </c>
-      <c r="K85" t="inlineStr">
-        <is>
-          <t>Civil Engineering</t>
-        </is>
-      </c>
-      <c r="L85" t="inlineStr">
-        <is>
-          <t>2026-2027</t>
-        </is>
-      </c>
-      <c r="M85" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N85" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
-      <c r="O85" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="P85" t="inlineStr">
-        <is>
-          <t>admitted</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>854461920326</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>Fatima Shaikh</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>2005-01-22</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>OBC-NCL</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>INDIAN</t>
-        </is>
-      </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>+91 74312 20961</t>
-        </is>
-      </c>
-      <c r="H86" t="inlineStr">
-        <is>
-          <t>student82@example.invalid</t>
-        </is>
-      </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>08551163422</t>
-        </is>
-      </c>
-      <c r="J86" t="inlineStr">
-        <is>
-          <t>B.Tech</t>
-        </is>
-      </c>
-      <c r="K86" t="inlineStr">
-        <is>
-          <t>Civil Engineering</t>
-        </is>
-      </c>
-      <c r="L86" t="inlineStr">
-        <is>
-          <t>2026-27</t>
-        </is>
-      </c>
-      <c r="M86" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N86" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
-      <c r="O86" t="inlineStr">
-        <is>
-          <t>04.08.2026</t>
-        </is>
-      </c>
-      <c r="P86" t="inlineStr">
-        <is>
-          <t>Admitted</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr"/>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>TOTAL = 83</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr"/>
-      <c r="D87" t="inlineStr"/>
-      <c r="E87" t="inlineStr"/>
-      <c r="F87" t="inlineStr"/>
-      <c r="G87" t="inlineStr"/>
-      <c r="H87" t="inlineStr"/>
-      <c r="I87" t="inlineStr"/>
-      <c r="J87" t="inlineStr"/>
-      <c r="K87" t="inlineStr"/>
-      <c r="L87" t="inlineStr"/>
-      <c r="M87" t="inlineStr"/>
-      <c r="N87" t="inlineStr"/>
-      <c r="O87" t="inlineStr"/>
-      <c r="P87" t="inlineStr"/>
+          <t>TOTAL = 63</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" t="inlineStr"/>
+      <c r="O67" t="inlineStr"/>
+      <c r="P67" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>